<commit_message>
Rebuild photographed forms as line art plus reliable text
Pages with many ruled boxes (e.g. a T4 slip) become one transparent
picture of the form's rules and print, with each recognized line placed
as an exact text box on top (Word text boxes, PowerPoint shapes, Excel
drawing shapes). Text is made editable only when it reads reliably:
spelled correctly in English or French, or confirmed by a second reading
for larger entries; anything else stays in the picture as printed, and
the picture loses exactly the ink of the text drawn over it.

Also: flattening keeps the paper's true aspect (Letter/A4 snap), wood
desks no longer pass as paper when extending to edges, and false rules
inside bold text are ignored.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2KPqXq9Whv7eR2vrvkBWC
</commit_message>
<xml_diff>
--- a/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
+++ b/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
@@ -17,6 +17,19 @@
       <family val="2"/>
     </font>
     <font>
+      <u/>
+      <sz val="12.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="27.5"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -37,19 +50,6 @@
     </font>
     <font>
       <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -133,18 +133,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -251,7 +251,7 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>260819</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>88708</xdr:rowOff>
+      <xdr:rowOff>88716</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="789908" cy="44712"/>
     <xdr:pic>
@@ -293,8 +293,8 @@
     <col min="2" max="2" width="0.57" customWidth="1"/>
     <col min="3" max="3" width="1.52" customWidth="1"/>
     <col min="4" max="4" width="22.09" customWidth="1"/>
-    <col min="5" max="5" width="16.08" customWidth="1"/>
-    <col min="6" max="6" width="20.05" customWidth="1"/>
+    <col min="5" max="5" width="16.11" customWidth="1"/>
+    <col min="6" max="6" width="20.02" customWidth="1"/>
     <col min="7" max="7" width="7.00" customWidth="1"/>
     <col min="8" max="8" width="11.52" customWidth="1"/>
     <col min="9" max="9" width="2.02" customWidth="1"/>
@@ -302,14 +302,14 @@
   <sheetData>
     <row r="1" ht="38.37" customHeight="1"/>
     <row r="2" ht="33.00" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">MYRIAD</t>
         </is>
       </c>
     </row>
     <row r="3" ht="9.66" customHeight="1">
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">HEART OF BURQUITLAM</t>
         </is>
@@ -317,7 +317,7 @@
     </row>
     <row r="4" ht="67.03" customHeight="1"/>
     <row r="5" ht="17.40" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Myriad - Prices at a Glance</t>
         </is>
@@ -325,7 +325,7 @@
     </row>
     <row r="6" ht="8.31" customHeight="1"/>
     <row r="7" ht="12.00" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">October 2021</t>
         </is>
@@ -333,200 +333,200 @@
     </row>
     <row r="8" ht="34.28" customHeight="1"/>
     <row r="9" ht="25.25" customHeight="1">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Suite Type</t>
         </is>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Plan</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Square Feet</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Starting From</t>
         </is>
       </c>
-      <c r="H9" s="5"/>
+      <c r="H9" s="1"/>
     </row>
     <row r="10" ht="24.86" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">One Bedroom</t>
         </is>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">AT*</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">476-479</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">476 - 479</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$449,900</t>
         </is>
       </c>
-      <c r="H10" s="6"/>
+      <c r="H10" s="2"/>
     </row>
     <row r="11" ht="21.85" customHeight="1">
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">B1 - B7</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">518 - 689</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$499,900</t>
         </is>
       </c>
-      <c r="H11" s="6"/>
-    </row>
-    <row r="12" ht="21.93" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" ht="21.97" customHeight="1">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">One Bedroom + Den</t>
         </is>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">C1 - C6</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">644-769</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">644 - 769</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$599,900</t>
         </is>
       </c>
-      <c r="H12" s="6"/>
-    </row>
-    <row r="13" ht="23.04" customHeight="1">
-      <c r="B13" s="6" t="inlineStr">
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" ht="23.16" customHeight="1">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Two Bedroom</t>
         </is>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">D1 - D7</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">801-989</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">801 - 989</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$729,900</t>
         </is>
       </c>
-      <c r="H13" s="6"/>
-    </row>
-    <row r="14" ht="24.76" customHeight="1">
-      <c r="B14" s="6" t="inlineStr">
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" ht="24.50" customHeight="1">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Two Bedroom + Den</t>
         </is>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">E1 - E7</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">834 - 1,062</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$749,900</t>
         </is>
       </c>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" ht="24.43" customHeight="1">
-      <c r="B15" s="6" t="inlineStr">
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" ht="24.53" customHeight="1">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Three Bedroom</t>
         </is>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">F11</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F1</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1,023</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$929,900</t>
         </is>
       </c>
-      <c r="H15" s="6"/>
+      <c r="H15" s="2"/>
     </row>
     <row r="16" ht="21.03" customHeight="1">
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Townhomes</t>
         </is>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TH1- TH4</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TH1 - TH4</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1,338 - 1,553</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$1,249,900</t>
         </is>
       </c>
-      <c r="H16" s="6"/>
+      <c r="H16" s="2"/>
     </row>
     <row r="17" ht="36.02" customHeight="1"/>
     <row r="18" ht="12.00" customHeight="1">
@@ -568,17 +568,16 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="2.00" customHeight="1"/>
-    <row r="28" ht="12.00" customHeight="1">
-      <c r="D28" s="7" t="inlineStr">
+    <row r="27" ht="12.11" customHeight="1">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 730 days.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="2.08" customHeight="1"/>
-    <row r="30" ht="12.60" customHeight="1">
-      <c r="D30" s="8" t="inlineStr">
+    <row r="28" ht="2.66" customHeight="1"/>
+    <row r="29" ht="12.60" customHeight="1">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -611,44 +610,43 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="56.61" customHeight="1"/>
-    <row r="32" ht="7.67" customHeight="1">
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prices do not include GST, may change without notice and are subject to availability. Sulte sizes may vary on final Strata Plan. Concert reserves the right to</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="6.89" customHeight="1">
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">make modifications and changes to floorplans, project design, specifications and features. October 2021. CONCERT REALTY SERVICES LTD. E. &amp;O.E.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="54.63" customHeight="1"/>
-    <row r="35" ht="9.79" customHeight="1">
-      <c r="B35" s="12" t="inlineStr">
+    <row r="30" ht="57.19" customHeight="1"/>
+    <row r="31" ht="7.67" customHeight="1">
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rices do not include GST, may change without notice and are subject to availability. Sulte sizes may vary on final Strata Plan. Concert reserves the right t</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="6.31" customHeight="1">
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">make modifications and changes to floorplans, project design, specifications and features. October 2021. CONCERT REALTY SERVICES LTD. E.&amp;O.E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="54.34" customHeight="1"/>
+    <row r="34" ht="10.36" customHeight="1">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">MyriadbyConcert.com</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="9.79" customHeight="1">
-      <c r="B36" s="13" t="inlineStr">
+    <row r="35" ht="10.36" customHeight="1">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">101 - 511 Clarke Road, Coquitlam, BC V3J 0J1</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="2.00" customHeight="1"/>
-    <row r="38" ht="9.60" customHeight="1">
-      <c r="B38" s="14" t="inlineStr">
+    <row r="36" ht="9.98" customHeight="1">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">604.335.0696 | Admin.Myriad@ConcertProperties.com</t>
         </is>
       </c>
-      <c r="H38" s="15" t="inlineStr">
+      <c r="H36" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">CONCERT®</t>
         </is>
@@ -656,10 +654,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A7:I7"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="B10:D10"/>
@@ -676,19 +670,23 @@
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="G16:H16"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="D20:I20"/>
     <mergeCell ref="D22:I22"/>
     <mergeCell ref="D24:I24"/>
     <mergeCell ref="D26:I26"/>
-    <mergeCell ref="D28:I28"/>
-    <mergeCell ref="D30:I30"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="B31:I31"/>
     <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B34:I34"/>
     <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="H36:I36"/>
   </mergeCells>
   <pageMargins left="0.46" right="1.03" top="0.29" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="1" orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Convert & read fixes from corpus testing; paywall colours; rename to FoldScan
- Office: keep recognized lines together (CJK interleaving), two-column pages
  as Word columns, outline-only tables rebuilt from aligned columns, wrapped
  row labels, spaces between columns, no tables from column prose, XML-safe
  text, sideways pages turned upright, small images enlarged, bold calibrated
  (incl. CJK, local light).
- Math: tolerant solver for photographed sheets (numbering, =, superscripts,
  √, x/÷), never merges "2 57" into 257.
- Photo translation: clamp edge boxes, light text on dark/colored signs.
- ConvertCorpusTests harness (private corpus, skipped when absent).
- Paywall: each slide its own stage colour. Extract text glyph square.
- App name FoldScan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2KPqXq9Whv7eR2vrvkBWC
</commit_message>
<xml_diff>
--- a/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
+++ b/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -30,6 +30,13 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="12.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="27.5"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -49,6 +56,13 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -98,6 +112,7 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
       <sz val="14.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -124,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -139,16 +154,13 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -169,6 +181,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -302,14 +320,14 @@
   <sheetData>
     <row r="1" ht="38.37" customHeight="1"/>
     <row r="2" ht="33.00" customHeight="1">
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">MYRIAD</t>
         </is>
       </c>
     </row>
     <row r="3" ht="9.66" customHeight="1">
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">HEART OF BURQUITLAM</t>
         </is>
@@ -317,7 +335,7 @@
     </row>
     <row r="4" ht="67.03" customHeight="1"/>
     <row r="5" ht="17.40" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Myriad - Prices at a Glance</t>
         </is>
@@ -325,7 +343,7 @@
     </row>
     <row r="6" ht="8.31" customHeight="1"/>
     <row r="7" ht="12.00" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">October 2021</t>
         </is>
@@ -365,14 +383,14 @@
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">AT*</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">476 - 479</t>
+          <t xml:space="preserve">476-479</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -393,7 +411,25 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">518 - 689</t>
+          <r>
+            <rPr>
+              <sz val="12.0"/>
+              <color rgb="FF000000"/>
+              <rFont val="Arial"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">518 -</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12.0"/>
+              <color rgb="FF000000"/>
+              <rFont val="Arial"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve"> 689</t>
+          </r>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -418,7 +454,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">644 - 769</t>
+          <t xml:space="preserve">644-769</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -443,7 +479,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">801 - 989</t>
+          <t xml:space="preserve">801-989</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -468,7 +504,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">834 - 1,062</t>
+          <t xml:space="preserve">834-1,062</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -518,7 +554,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1,338 - 1,553</t>
+          <t xml:space="preserve">1,338-1,553</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -530,7 +566,7 @@
     </row>
     <row r="17" ht="36.02" customHeight="1"/>
     <row r="18" ht="12.00" customHeight="1">
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Deposit Structure:</t>
         </is>
@@ -538,7 +574,7 @@
     </row>
     <row r="19" ht="10.12" customHeight="1"/>
     <row r="20" ht="12.60" customHeight="1">
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">•  Initial $10,000 bank draft due upon signing Offer to Purchase and Agreement Sale;</t>
         </is>
@@ -546,7 +582,7 @@
     </row>
     <row r="21" ht="2.00" customHeight="1"/>
     <row r="22" ht="12.00" customHeight="1">
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% within 7 days (less $10,000 initial deposit) upon signing;</t>
         </is>
@@ -554,7 +590,7 @@
     </row>
     <row r="23" ht="2.00" customHeight="1"/>
     <row r="24" ht="11.40" customHeight="1">
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 180 days;</t>
         </is>
@@ -562,14 +598,14 @@
     </row>
     <row r="25" ht="2.00" customHeight="1"/>
     <row r="26" ht="12.00" customHeight="1">
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 365 days;</t>
         </is>
       </c>
     </row>
     <row r="27" ht="12.11" customHeight="1">
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 730 days.</t>
         </is>
@@ -577,7 +613,7 @@
     </row>
     <row r="28" ht="2.66" customHeight="1"/>
     <row r="29" ht="12.60" customHeight="1">
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -612,14 +648,14 @@
     </row>
     <row r="30" ht="57.19" customHeight="1"/>
     <row r="31" ht="7.67" customHeight="1">
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">rices do not include GST, may change without notice and are subject to availability. Sulte sizes may vary on final Strata Plan. Concert reserves the right t</t>
         </is>
       </c>
     </row>
     <row r="32" ht="6.31" customHeight="1">
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">make modifications and changes to floorplans, project design, specifications and features. October 2021. CONCERT REALTY SERVICES LTD. E.&amp;O.E.</t>
         </is>
@@ -627,26 +663,26 @@
     </row>
     <row r="33" ht="54.34" customHeight="1"/>
     <row r="34" ht="10.36" customHeight="1">
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">MyriadbyConcert.com</t>
         </is>
       </c>
     </row>
     <row r="35" ht="10.36" customHeight="1">
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">101 - 511 Clarke Road, Coquitlam, BC V3J 0J1</t>
         </is>
       </c>
     </row>
     <row r="36" ht="9.98" customHeight="1">
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B36" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">604.335.0696 | Admin.Myriad@ConcertProperties.com</t>
         </is>
       </c>
-      <c r="H36" s="15" t="inlineStr">
+      <c r="H36" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">CONCERT®</t>
         </is>

</xml_diff>

<commit_message>
Page frame and heading bars in Office export, receipt fixes, UVDoc benchmark, flatten by surface length
- Page-wide frame becomes a Word page border; dark and gray heading bars become paragraph shading
- Fix out-of-range read in Ink.fill (crash on pages with text near the edge)
- Pictures made mostly of recognized words keep only the unread ink (no doubled receipt totals)
- One-line paragraphs no taller than the room to the next line; short words capped by width
- Accept confident document segmentation on heavily printed pages; prefer the sheet over a printed rectangle inside it
- Snap aspect to the nearest paper size; lay out the flattened page by surface arc length
- UVDoc benchmark test and scorer support

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2KPqXq9Whv7eR2vrvkBWC
</commit_message>
<xml_diff>
--- a/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
+++ b/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
@@ -37,7 +37,7 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="27.5"/>
+      <sz val="21.7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -266,8 +266,8 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>260819</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>495556</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>88716</xdr:rowOff>
     </xdr:from>
@@ -308,14 +308,11 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.84" customWidth="1"/>
-    <col min="2" max="2" width="0.57" customWidth="1"/>
-    <col min="3" max="3" width="1.52" customWidth="1"/>
-    <col min="4" max="4" width="22.09" customWidth="1"/>
-    <col min="5" max="5" width="16.11" customWidth="1"/>
-    <col min="6" max="6" width="20.02" customWidth="1"/>
-    <col min="7" max="7" width="7.00" customWidth="1"/>
-    <col min="8" max="8" width="11.52" customWidth="1"/>
-    <col min="9" max="9" width="2.02" customWidth="1"/>
+    <col min="2" max="2" width="25.61" customWidth="1"/>
+    <col min="3" max="3" width="16.11" customWidth="1"/>
+    <col min="4" max="4" width="20.02" customWidth="1"/>
+    <col min="5" max="5" width="19.24" customWidth="1"/>
+    <col min="6" max="6" width="2.02" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="38.37" customHeight="1"/>
@@ -327,7 +324,7 @@
       </c>
     </row>
     <row r="3" ht="9.66" customHeight="1">
-      <c r="C3" s="5" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">HEART OF BURQUITLAM</t>
         </is>
@@ -356,24 +353,21 @@
           <t xml:space="preserve">Suite Type</t>
         </is>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plan</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square Feet</t>
+        </is>
+      </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plan</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Square Feet</t>
-        </is>
-      </c>
-      <c r="G9" s="1" t="inlineStr">
-        <is>
           <t xml:space="preserve">Starting From</t>
         </is>
       </c>
-      <c r="H9" s="1"/>
     </row>
     <row r="10" ht="24.86" customHeight="1">
       <c r="B10" s="2" t="inlineStr">
@@ -381,35 +375,30 @@
           <t xml:space="preserve">One Bedroom</t>
         </is>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">AT*</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">476-479</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$449,900</t>
         </is>
       </c>
-      <c r="H10" s="2"/>
     </row>
     <row r="11" ht="21.85" customHeight="1">
       <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">B1 - B7</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -432,12 +421,11 @@
           </r>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$499,900</t>
         </is>
       </c>
-      <c r="H11" s="2"/>
     </row>
     <row r="12" ht="21.97" customHeight="1">
       <c r="B12" s="2" t="inlineStr">
@@ -445,24 +433,21 @@
           <t xml:space="preserve">One Bedroom + Den</t>
         </is>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C1 - C6</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">644-769</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C1 - C6</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">644-769</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">$599,900</t>
         </is>
       </c>
-      <c r="H12" s="2"/>
     </row>
     <row r="13" ht="23.16" customHeight="1">
       <c r="B13" s="2" t="inlineStr">
@@ -470,24 +455,21 @@
           <t xml:space="preserve">Two Bedroom</t>
         </is>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D1 - D7</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">801-989</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">D1 - D7</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">801-989</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">$729,900</t>
         </is>
       </c>
-      <c r="H13" s="2"/>
     </row>
     <row r="14" ht="24.50" customHeight="1">
       <c r="B14" s="2" t="inlineStr">
@@ -495,24 +477,21 @@
           <t xml:space="preserve">Two Bedroom + Den</t>
         </is>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E1 - E7</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">834-1,062</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">E1 - E7</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">834-1,062</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">$749,900</t>
         </is>
       </c>
-      <c r="H14" s="2"/>
     </row>
     <row r="15" ht="24.53" customHeight="1">
       <c r="B15" s="2" t="inlineStr">
@@ -520,24 +499,21 @@
           <t xml:space="preserve">Three Bedroom</t>
         </is>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F1</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1,023</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">F1</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1,023</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">$929,900</t>
         </is>
       </c>
-      <c r="H15" s="2"/>
     </row>
     <row r="16" ht="21.03" customHeight="1">
       <c r="B16" s="2" t="inlineStr">
@@ -545,24 +521,21 @@
           <t xml:space="preserve">Townhomes</t>
         </is>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TH1 - TH4</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1,338-1,553</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH1 - TH4</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1,338-1,553</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">$1,249,900</t>
         </is>
       </c>
-      <c r="H16" s="2"/>
     </row>
     <row r="17" ht="36.02" customHeight="1"/>
     <row r="18" ht="12.00" customHeight="1">
@@ -574,7 +547,7 @@
     </row>
     <row r="19" ht="10.12" customHeight="1"/>
     <row r="20" ht="12.60" customHeight="1">
-      <c r="D20" s="9" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">•  Initial $10,000 bank draft due upon signing Offer to Purchase and Agreement Sale;</t>
         </is>
@@ -582,7 +555,7 @@
     </row>
     <row r="21" ht="2.00" customHeight="1"/>
     <row r="22" ht="12.00" customHeight="1">
-      <c r="D22" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% within 7 days (less $10,000 initial deposit) upon signing;</t>
         </is>
@@ -590,7 +563,7 @@
     </row>
     <row r="23" ht="2.00" customHeight="1"/>
     <row r="24" ht="11.40" customHeight="1">
-      <c r="D24" s="10" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 180 days;</t>
         </is>
@@ -598,14 +571,14 @@
     </row>
     <row r="25" ht="2.00" customHeight="1"/>
     <row r="26" ht="12.00" customHeight="1">
-      <c r="D26" s="8" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 365 days;</t>
         </is>
       </c>
     </row>
     <row r="27" ht="12.11" customHeight="1">
-      <c r="D27" s="8" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 730 days.</t>
         </is>
@@ -613,7 +586,7 @@
     </row>
     <row r="28" ht="2.66" customHeight="1"/>
     <row r="29" ht="12.60" customHeight="1">
-      <c r="D29" s="9" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -682,47 +655,31 @@
           <t xml:space="preserve">604.335.0696 | Admin.Myriad@ConcertProperties.com</t>
         </is>
       </c>
-      <c r="H36" s="16" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">CONCERT®</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C3:I3"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="B18:I18"/>
-    <mergeCell ref="D20:I20"/>
-    <mergeCell ref="D22:I22"/>
-    <mergeCell ref="D24:I24"/>
-    <mergeCell ref="D26:I26"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="D29:I29"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B36:G36"/>
-    <mergeCell ref="H36:I36"/>
+  <mergeCells count="17">
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="E36:F36"/>
   </mergeCells>
   <pageMargins left="0.46" right="1.03" top="0.29" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="1" orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Sharper scans: 48 MP capture in good light, supersampled clarity step
- Camera: good light captures at the sensor's full 48 MP and decodes
  straight to ~24 MP with ImageIO (orientation applied); dim light keeps
  the ~12 MP three-frame burst.
- Clarity: pages with a long side under 3600 px run the stroke step at
  up to 2x and scale back, so letter edges stay antialiased instead of
  snapping to whole pixels. Page size and coordinates are unchanged.
- Ink ramp (0.18, 0.55) -> (0.14, 0.65); 0.12-0.8 loses thin printed
  checkboxes on the Notice sample.
- Sharpness test reads the phone scan with its saved crop.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2KPqXq9Whv7eR2vrvkBWC
</commit_message>
<xml_diff>
--- a/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
+++ b/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="17">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -43,7 +43,7 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9.0"/>
+      <sz val="7.5"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -95,18 +95,6 @@
     <font>
       <b/>
       <sz val="7.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="7.5"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -139,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -181,12 +169,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -205,7 +187,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="491830" cy="59616"/>
+    <xdr:ext cx="476926" cy="59616"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 1"/>
@@ -222,7 +204,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="491830" cy="59616"/>
+          <a:ext cx="476926" cy="59616"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -264,39 +246,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>495556</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>88716</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="789908" cy="44712"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="789908" cy="44712"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -307,10 +256,10 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.84" customWidth="1"/>
-    <col min="2" max="2" width="25.61" customWidth="1"/>
-    <col min="3" max="3" width="16.11" customWidth="1"/>
-    <col min="4" max="4" width="20.02" customWidth="1"/>
+    <col min="1" max="1" width="8.51" customWidth="1"/>
+    <col min="2" max="2" width="25.94" customWidth="1"/>
+    <col min="3" max="3" width="16.08" customWidth="1"/>
+    <col min="4" max="4" width="20.05" customWidth="1"/>
     <col min="5" max="5" width="19.24" customWidth="1"/>
     <col min="6" max="6" width="2.02" customWidth="1"/>
   </cols>
@@ -323,14 +272,14 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="9.66" customHeight="1">
+    <row r="3" ht="8.76" customHeight="1">
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">HEART OF BURQUITLAM</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="67.03" customHeight="1"/>
+    <row r="4" ht="67.93" customHeight="1"/>
     <row r="5" ht="17.40" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -342,12 +291,30 @@
     <row r="7" ht="12.00" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">October 2021</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34.28" customHeight="1"/>
-    <row r="9" ht="25.25" customHeight="1">
+          <r>
+            <rPr>
+              <b/>
+              <sz val="10.0"/>
+              <color rgb="FF000000"/>
+              <rFont val="Arial"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve">October</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="10.0"/>
+              <color rgb="FF000000"/>
+              <rFont val="Arial"/>
+              <family val="2"/>
+            </rPr>
+            <t xml:space="preserve"> 2021</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34.76" customHeight="1"/>
+    <row r="9" ht="24.77" customHeight="1">
       <c r="B9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Suite Type</t>
@@ -391,7 +358,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="21.85" customHeight="1">
+    <row r="11" ht="21.83" customHeight="1">
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -427,7 +394,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="21.97" customHeight="1">
+    <row r="12" ht="22.02" customHeight="1">
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">One Bedroom + Den</t>
@@ -449,7 +416,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="23.16" customHeight="1">
+    <row r="13" ht="23.15" customHeight="1">
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Two Bedroom</t>
@@ -471,7 +438,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="24.50" customHeight="1">
+    <row r="14" ht="24.48" customHeight="1">
       <c r="B14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Two Bedroom + Den</t>
@@ -577,16 +544,17 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="12.11" customHeight="1">
-      <c r="B27" s="8" t="inlineStr">
+    <row r="27" ht="2.00" customHeight="1"/>
+    <row r="28" ht="12.00" customHeight="1">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 730 days.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="2.66" customHeight="1"/>
-    <row r="29" ht="12.60" customHeight="1">
-      <c r="B29" s="9" t="inlineStr">
+    <row r="29" ht="2.08" customHeight="1"/>
+    <row r="30" ht="12.60" customHeight="1">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -619,43 +587,44 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="57.19" customHeight="1"/>
-    <row r="31" ht="7.67" customHeight="1">
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rices do not include GST, may change without notice and are subject to availability. Sulte sizes may vary on final Strata Plan. Concert reserves the right t</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="6.31" customHeight="1">
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">make modifications and changes to floorplans, project design, specifications and features. October 2021. CONCERT REALTY SERVICES LTD. E.&amp;O.E.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="54.34" customHeight="1"/>
-    <row r="34" ht="10.36" customHeight="1">
-      <c r="B34" s="13" t="inlineStr">
+    <row r="31" ht="57.19" customHeight="1"/>
+    <row r="32" ht="7.67" customHeight="1">
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prices do not include GST, may change without notice and are subject to availability. Sulte sizes may vary on final Strata Plan. Concert reserves the right to</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="6.31" customHeight="1">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nake modifications and changes to floorplans, project design, specifications and features. October 2021. CONCERT REALTY SERVICES LTD. E.8O.!</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="54.63" customHeight="1"/>
+    <row r="35" ht="9.79" customHeight="1">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">MyriadbyConcert.com</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="10.36" customHeight="1">
-      <c r="B35" s="14" t="inlineStr">
+    <row r="36" ht="9.79" customHeight="1">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">101 - 511 Clarke Road, Coquitlam, BC V3J 0J1</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="9.98" customHeight="1">
-      <c r="B36" s="15" t="inlineStr">
+    <row r="37" ht="2.00" customHeight="1"/>
+    <row r="38" ht="9.00" customHeight="1">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">604.335.0696 | Admin.Myriad@ConcertProperties.com</t>
         </is>
       </c>
-      <c r="E36" s="16" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">CONCERT®</t>
         </is>
@@ -672,14 +641,14 @@
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B30:F30"/>
     <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B33:F33"/>
     <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="E38:F38"/>
   </mergeCells>
   <pageMargins left="0.46" right="1.03" top="0.29" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="1" orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Packing list: page frame, banded tables, numbered columns; flatter, crisper scan
- Layout: the page frame gives its sides back as cell walls; collinear rule
  pieces join; tables split into bands of matching walls; empty merged cells
  are split along shared row/column lines; a logo bar in a cell becomes a picture.
- Re-reading: numbered columns are filled and corrected from their sequence;
  a sign never turns into a letter, and a capital never into its small letter.
- Excel: row edges from every band; table cells shrink to fit.
- Scan: the flatten mesh samples through a homography plus offsets (straight
  rules); the paper background is lifted to white so text reads clearly.
- UI test: settle the Welcome to Pro card before opening the saved document.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2KPqXq9Whv7eR2vrvkBWC
</commit_message>
<xml_diff>
--- a/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
+++ b/ios/Verification/office-layout/OfficeSamplePhoto.xlsx
@@ -37,7 +37,7 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="21.7"/>
+      <sz val="21.4"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -130,13 +130,13 @@
   <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -265,21 +265,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="38.37" customHeight="1"/>
-    <row r="2" ht="33.00" customHeight="1">
+    <row r="2" ht="32.54" customHeight="1">
       <c r="B2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">MYRIAD</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="8.76" customHeight="1">
+    <row r="3" ht="9.00" customHeight="1">
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">HEART OF BURQUITLAM</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="67.93" customHeight="1"/>
+    <row r="4" ht="67.00" customHeight="1"/>
     <row r="5" ht="17.40" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -287,7 +287,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="8.31" customHeight="1"/>
+    <row r="6" ht="8.90" customHeight="1"/>
     <row r="7" ht="12.00" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
@@ -313,8 +313,8 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="34.76" customHeight="1"/>
-    <row r="9" ht="24.77" customHeight="1">
+    <row r="8" ht="34.39" customHeight="1"/>
+    <row r="9" ht="25.12" customHeight="1">
       <c r="B9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Suite Type</t>
@@ -336,7 +336,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24.86" customHeight="1">
+    <row r="10" ht="25.58" customHeight="1">
       <c r="B10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">One Bedroom</t>
@@ -358,7 +358,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="21.83" customHeight="1">
+    <row r="11" ht="22.19" customHeight="1">
       <c r="B11" s="2"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -394,7 +394,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22.02" customHeight="1">
+    <row r="12" ht="21.47" customHeight="1">
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">One Bedroom + Den</t>
@@ -416,7 +416,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="23.15" customHeight="1">
+    <row r="13" ht="22.66" customHeight="1">
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Two Bedroom</t>
@@ -438,7 +438,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="24.48" customHeight="1">
+    <row r="14" ht="25.14" customHeight="1">
       <c r="B14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Two Bedroom + Den</t>
@@ -460,7 +460,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24.53" customHeight="1">
+    <row r="15" ht="24.67" customHeight="1">
       <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Three Bedroom</t>
@@ -482,7 +482,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="21.03" customHeight="1">
+    <row r="16" ht="20.36" customHeight="1">
       <c r="B16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Townhomes</t>
@@ -504,7 +504,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="36.02" customHeight="1"/>
+    <row r="17" ht="36.45" customHeight="1"/>
     <row r="18" ht="12.00" customHeight="1">
       <c r="B18" s="8" t="inlineStr">
         <is>
@@ -512,7 +512,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="10.12" customHeight="1"/>
+    <row r="19" ht="10.42" customHeight="1"/>
     <row r="20" ht="12.60" customHeight="1">
       <c r="B20" s="9" t="inlineStr">
         <is>
@@ -520,41 +520,37 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="2.00" customHeight="1"/>
-    <row r="22" ht="12.00" customHeight="1">
+    <row r="21" ht="2.44" customHeight="1"/>
+    <row r="22" ht="10.79" customHeight="1">
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">•  5% within 7 days (less $10,000 initial deposit) upon signing;</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="2.00" customHeight="1"/>
-    <row r="24" ht="11.40" customHeight="1">
-      <c r="B24" s="10" t="inlineStr">
+          <t xml:space="preserve">pe</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="12.95" customHeight="1">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 180 days;</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="2.00" customHeight="1"/>
-    <row r="26" ht="12.00" customHeight="1">
-      <c r="B26" s="8" t="inlineStr">
+    <row r="24" ht="13.53" customHeight="1">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 365 days;</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="2.00" customHeight="1"/>
-    <row r="28" ht="12.00" customHeight="1">
-      <c r="B28" s="8" t="inlineStr">
+    <row r="25" ht="12.69" customHeight="1">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">•  5% in 730 days.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="2.08" customHeight="1"/>
-    <row r="30" ht="12.60" customHeight="1">
-      <c r="B30" s="9" t="inlineStr">
+    <row r="26" ht="14.68" customHeight="1">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -587,46 +583,45 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="57.19" customHeight="1"/>
-    <row r="32" ht="7.67" customHeight="1">
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Prices do not include GST, may change without notice and are subject to availability. Sulte sizes may vary on final Strata Plan. Concert reserves the right to</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="6.31" customHeight="1">
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nake modifications and changes to floorplans, project design, specifications and features. October 2021. CONCERT REALTY SERVICES LTD. E.8O.!</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="54.63" customHeight="1"/>
-    <row r="35" ht="9.79" customHeight="1">
-      <c r="B35" s="13" t="inlineStr">
+    <row r="27" ht="57.18" customHeight="1"/>
+    <row r="28" ht="6.89" customHeight="1">
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prices do not include GST, may change without notice and are subject to availability. Suite sizes may vary on final Strata Plan. Concert reserves the right to</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="7.67" customHeight="1">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">make modifications and changes to floorplans, project design, specifications and features. October 2021. CONCERT REALTY SERVICES LTD. E.&amp;O.E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="54.35" customHeight="1"/>
+    <row r="31" ht="9.21" customHeight="1">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">MyriadbyConcert.com</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="9.79" customHeight="1">
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">101 - 511 Clarke Road, Coquitlam, BC V3J 0J1</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="2.00" customHeight="1"/>
-    <row r="38" ht="9.00" customHeight="1">
-      <c r="B38" s="5" t="inlineStr">
+    <row r="32" ht="9.21" customHeight="1">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">101 - 511 Clarke Road, Coquitlam, BC V3J 0/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="10.83" customHeight="1">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">604.335.0696 | Admin.Myriad@ConcertProperties.com</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONCERT®</t>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONCERT'</t>
         </is>
       </c>
     </row>
@@ -639,16 +634,16 @@
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B23:F23"/>
     <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B25:F25"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B31:F31"/>
     <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="E33:F33"/>
   </mergeCells>
   <pageMargins left="0.46" right="1.03" top="0.29" bottom="0.3" header="0" footer="0"/>
   <pageSetup paperSize="1" orientation="portrait" fitToWidth="1" fitToHeight="0"/>

</xml_diff>